<commit_message>
added product page and tests
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginData.xlsx
+++ b/src/test/resources/testdata/LoginData.xlsx
@@ -8,13 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Selenium_projects\SauceDemo_Automation\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DB3F5198-85E8-4127-B2EA-6142A032DD34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21FB766C-462B-4FF1-BCE4-642B19BA9AFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{E635F91A-BCC6-4F84-AD84-A5C24D3DB13A}"/>
   </bookViews>
   <sheets>
     <sheet name="Valid_data" sheetId="1" r:id="rId1"/>
-    <sheet name="Invalid_data" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>Username</t>
   </si>
@@ -53,18 +52,6 @@
   </si>
   <si>
     <t>performance_glitch_user</t>
-  </si>
-  <si>
-    <t>abc</t>
-  </si>
-  <si>
-    <t>invalid_test</t>
-  </si>
-  <si>
-    <t>invalid_username</t>
-  </si>
-  <si>
-    <t>invalid_passw</t>
   </si>
 </sst>
 </file>
@@ -461,54 +448,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7849EA1-5342-49D9-A929-664CC7FDA94E}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>